<commit_message>
fix fiscal year 2027 bug
</commit_message>
<xml_diff>
--- a/inst/extdata/region/2026-08-12/wb_projects_gov_menaap.xlsx
+++ b/inst/extdata/region/2026-08-12/wb_projects_gov_menaap.xlsx
@@ -1155,7 +1155,9 @@
       <c r="T7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U7" s="2"/>
+      <c r="U7" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="V7" s="2" t="s">
         <v>35</v>
       </c>
@@ -1215,7 +1217,9 @@
       <c r="T8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="U8" s="2"/>
+      <c r="U8" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="V8" s="2" t="s">
         <v>35</v>
       </c>

</xml_diff>